<commit_message>
Finalização da parte 3 do curso de HTML5 e CSS3
</commit_message>
<xml_diff>
--- a/Plano de estudos - Alura.xlsx
+++ b/Plano de estudos - Alura.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SaraSampaio\Documents\Alura\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SaraSampaio\Documents\Cursos_Alura\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A245388B-FC61-40AF-B269-1B77A12E8DE1}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DFAEDA10-D981-41B7-A667-8FF188339FAE}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{8BCCBAC8-5B76-435E-AC96-991D0622A05E}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="47">
   <si>
     <t>PLANO DE ESTUDOS ALURA</t>
   </si>
@@ -163,6 +163,9 @@
   </si>
   <si>
     <t>Curso Web Design Responsivo: Páginas que se adaptam do mobile ao desk</t>
+  </si>
+  <si>
+    <t>3h</t>
   </si>
 </sst>
 </file>
@@ -329,7 +332,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="52">
+  <cellXfs count="53">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -441,6 +444,18 @@
     <xf numFmtId="16" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="16" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="16" fontId="3" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="16" fontId="5" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -451,15 +466,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="16" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="16" fontId="3" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="16" fontId="5" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -791,14 +797,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="21" x14ac:dyDescent="0.35">
-      <c r="A1" s="45" t="s">
+      <c r="A1" s="49" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="45"/>
-      <c r="C1" s="45"/>
-      <c r="D1" s="45"/>
-      <c r="E1" s="45"/>
-      <c r="F1" s="45"/>
+      <c r="B1" s="49"/>
+      <c r="C1" s="49"/>
+      <c r="D1" s="49"/>
+      <c r="E1" s="49"/>
+      <c r="F1" s="49"/>
     </row>
     <row r="2" spans="1:6" ht="31" x14ac:dyDescent="0.35">
       <c r="A2" s="11" t="s">
@@ -821,7 +827,7 @@
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A3" s="46" t="s">
+      <c r="A3" s="50" t="s">
         <v>1</v>
       </c>
       <c r="B3" s="19" t="s">
@@ -841,7 +847,7 @@
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A4" s="47" t="s">
+      <c r="A4" s="51" t="s">
         <v>1</v>
       </c>
       <c r="B4" s="20" t="s">
@@ -861,7 +867,7 @@
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A5" s="47" t="s">
+      <c r="A5" s="51" t="s">
         <v>1</v>
       </c>
       <c r="B5" s="39" t="s">
@@ -881,7 +887,7 @@
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A6" s="47" t="s">
+      <c r="A6" s="51" t="s">
         <v>1</v>
       </c>
       <c r="B6" s="16" t="s">
@@ -901,7 +907,7 @@
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A7" s="47" t="s">
+      <c r="A7" s="51" t="s">
         <v>1</v>
       </c>
       <c r="B7" s="17" t="s">
@@ -916,12 +922,12 @@
       <c r="E7" s="44">
         <v>44239</v>
       </c>
-      <c r="F7" s="51">
+      <c r="F7" s="48">
         <v>44244</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A8" s="48" t="s">
+      <c r="A8" s="52" t="s">
         <v>1</v>
       </c>
       <c r="B8" s="21" t="s">
@@ -933,15 +939,15 @@
       <c r="D8" s="13" t="s">
         <v>42</v>
       </c>
-      <c r="E8" s="49">
+      <c r="E8" s="46">
         <v>44244</v>
       </c>
-      <c r="F8" s="50">
+      <c r="F8" s="47">
         <v>44244</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A9" s="46" t="s">
+      <c r="A9" s="50" t="s">
         <v>17</v>
       </c>
       <c r="B9" s="39" t="s">
@@ -961,7 +967,7 @@
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A10" s="47" t="s">
+      <c r="A10" s="51" t="s">
         <v>17</v>
       </c>
       <c r="B10" s="16" t="s">
@@ -981,7 +987,7 @@
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A11" s="47" t="s">
+      <c r="A11" s="51" t="s">
         <v>17</v>
       </c>
       <c r="B11" s="20" t="s">
@@ -990,12 +996,18 @@
       <c r="C11" s="2">
         <v>8</v>
       </c>
-      <c r="D11" s="20"/>
-      <c r="E11" s="2"/>
-      <c r="F11" s="20"/>
+      <c r="D11" s="20" t="s">
+        <v>46</v>
+      </c>
+      <c r="E11" s="3">
+        <v>44247</v>
+      </c>
+      <c r="F11" s="15">
+        <v>44247</v>
+      </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A12" s="47" t="s">
+      <c r="A12" s="51" t="s">
         <v>17</v>
       </c>
       <c r="B12" s="20" t="s">
@@ -1004,12 +1016,12 @@
       <c r="C12" s="2">
         <v>8</v>
       </c>
-      <c r="D12" s="20"/>
+      <c r="D12" s="45"/>
       <c r="E12" s="2"/>
       <c r="F12" s="20"/>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A13" s="47" t="s">
+      <c r="A13" s="51" t="s">
         <v>17</v>
       </c>
       <c r="B13" s="17" t="s">
@@ -1024,12 +1036,12 @@
       <c r="E13" s="44">
         <v>44239</v>
       </c>
-      <c r="F13" s="51">
+      <c r="F13" s="48">
         <v>44244</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A14" s="47" t="s">
+      <c r="A14" s="51" t="s">
         <v>17</v>
       </c>
       <c r="B14" s="1" t="s">
@@ -1043,7 +1055,7 @@
       <c r="F14" s="20"/>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A15" s="47" t="s">
+      <c r="A15" s="51" t="s">
         <v>17</v>
       </c>
       <c r="B15" s="1" t="s">
@@ -1057,7 +1069,7 @@
       <c r="F15" s="20"/>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A16" s="47" t="s">
+      <c r="A16" s="51" t="s">
         <v>17</v>
       </c>
       <c r="B16" s="1" t="s">
@@ -1071,7 +1083,7 @@
       <c r="F16" s="20"/>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A17" s="48" t="s">
+      <c r="A17" s="52" t="s">
         <v>17</v>
       </c>
       <c r="B17" s="10" t="s">
@@ -1085,7 +1097,7 @@
       <c r="F17" s="21"/>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A18" s="46" t="s">
+      <c r="A18" s="50" t="s">
         <v>27</v>
       </c>
       <c r="B18" s="19" t="s">
@@ -1099,7 +1111,7 @@
       <c r="F18" s="23"/>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A19" s="47" t="s">
+      <c r="A19" s="51" t="s">
         <v>27</v>
       </c>
       <c r="B19" s="20" t="s">
@@ -1113,7 +1125,7 @@
       <c r="F19" s="24"/>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A20" s="47" t="s">
+      <c r="A20" s="51" t="s">
         <v>27</v>
       </c>
       <c r="B20" s="20" t="s">
@@ -1127,7 +1139,7 @@
       <c r="F20" s="24"/>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A21" s="47" t="s">
+      <c r="A21" s="51" t="s">
         <v>27</v>
       </c>
       <c r="B21" s="20" t="s">
@@ -1141,7 +1153,7 @@
       <c r="F21" s="24"/>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A22" s="47" t="s">
+      <c r="A22" s="51" t="s">
         <v>27</v>
       </c>
       <c r="B22" s="20" t="s">
@@ -1155,7 +1167,7 @@
       <c r="F22" s="24"/>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A23" s="47" t="s">
+      <c r="A23" s="51" t="s">
         <v>27</v>
       </c>
       <c r="B23" s="20" t="s">
@@ -1169,7 +1181,7 @@
       <c r="F23" s="24"/>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A24" s="47" t="s">
+      <c r="A24" s="51" t="s">
         <v>27</v>
       </c>
       <c r="B24" s="20" t="s">
@@ -1183,7 +1195,7 @@
       <c r="F24" s="24"/>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A25" s="47" t="s">
+      <c r="A25" s="51" t="s">
         <v>27</v>
       </c>
       <c r="B25" s="20" t="s">
@@ -1197,7 +1209,7 @@
       <c r="F25" s="24"/>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A26" s="48" t="s">
+      <c r="A26" s="52" t="s">
         <v>27</v>
       </c>
       <c r="B26" s="21" t="s">
@@ -1211,7 +1223,7 @@
       <c r="F26" s="25"/>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A27" s="46" t="s">
+      <c r="A27" s="50" t="s">
         <v>35</v>
       </c>
       <c r="B27" s="1" t="s">
@@ -1224,7 +1236,7 @@
       <c r="F27" s="30"/>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A28" s="47" t="s">
+      <c r="A28" s="51" t="s">
         <v>35</v>
       </c>
       <c r="B28" s="1" t="s">
@@ -1237,7 +1249,7 @@
       <c r="F28" s="31"/>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A29" s="47" t="s">
+      <c r="A29" s="51" t="s">
         <v>35</v>
       </c>
       <c r="B29" s="1" t="s">
@@ -1250,7 +1262,7 @@
       <c r="F29" s="31"/>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A30" s="47" t="s">
+      <c r="A30" s="51" t="s">
         <v>35</v>
       </c>
       <c r="B30" s="1" t="s">
@@ -1263,7 +1275,7 @@
       <c r="F30" s="31"/>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A31" s="47" t="s">
+      <c r="A31" s="51" t="s">
         <v>35</v>
       </c>
       <c r="B31" s="1" t="s">
@@ -1276,7 +1288,7 @@
       <c r="F31" s="31"/>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A32" s="47" t="s">
+      <c r="A32" s="51" t="s">
         <v>35</v>
       </c>
       <c r="B32" s="1" t="s">
@@ -1289,7 +1301,7 @@
       <c r="F32" s="31"/>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A33" s="48" t="s">
+      <c r="A33" s="52" t="s">
         <v>35</v>
       </c>
       <c r="B33" s="10" t="s">

</xml_diff>